<commit_message>
Tabla 3: quitar panel de brechas precio-costo (incoherente con subsidios)
El promedio de las brechas precio-costo sobre todos los país-años mezclaba
los que gravan (brecha positiva) con los que subsidian, dando un signo que
parecía contradecir el subsidio explícito del Panel A. La brecha es insumo
técnico del cálculo del subsidio, no necesita tabla propia. La Tabla 3 queda
con subsidios (explícito/implícito/total) + Brent, internamente coherente.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/tables/tab3_variables.xlsx
+++ b/outputs/tables/tab3_variables.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">Tabla 3. Estadística descriptiva del panel, por grupo de exposición fiscal</t>
   </si>
@@ -83,70 +83,7 @@
     <t xml:space="preserve">27</t>
   </si>
   <si>
-    <t xml:space="preserve">Panel B. Mecanismo de transmisión: brecha precio-costo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Brecha gasolina (USD/litro)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.29 (0.41)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.19 (0.36)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.41 (0.32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Brecha diésel (USD/litro)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.24 (0.32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.10 (0.38)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.33 (0.24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Brecha gas natural (USD/MMBtu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.10 (5.66)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.26 (3.58)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.46 (5.96)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Precio gasolina al consumidor (USD/litro)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.16 (0.42)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.67 (0.38)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.29 (0.32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Costo de suministro gasolina (USD/litro)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.87 (0.19)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.86 (0.17)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.88 (0.20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panel C. Choque: precio internacional del petróleo</t>
+    <t xml:space="preserve">Panel B. Choque: precio internacional del petróleo</t>
   </si>
   <si>
     <t xml:space="preserve">  Precio del Brent (USD/barril)</t>
@@ -158,18 +95,17 @@
     <t xml:space="preserve">—</t>
   </si>
   <si>
-    <t xml:space="preserve">Notas. Estadística descriptiva de las variables del análisis para el panel de 34 países de América Latina y el Caribe, 2015-2023. Cada celda reporta la media y, entre paréntesis, la desviación estándar de las observaciones país-año del grupo. El subsidio explícito es la brecha entre el precio al consumidor y el costo de suministro; el implícito añade las externalidades no internalizadas y el IVA no aplicado; el total es la suma de ambos. El subsidio implícito y el total tienen menor cobertura (no estimados para todos los país-año). El análisis del choque (Figuras 1 y 2) se concentra en el componente explícito por ser el más sensible al precio internacional en el corto plazo: reacciona de forma directa cuando el alza del costo de suministro no se traslada al precio al consumidor. El implícito depende del volumen consumido y de parámetros de daño ambiental, no del precio del petróleo, por lo que apenas responde al choque en el corto plazo. Las brechas precio-costo (Panel B) son el canal de transmisión: una brecha negativa indica precio al consumidor por debajo del costo de suministro, es decir, subsidio. El precio del Brent (Panel C) es la serie internacional, común a todos los países cada año, por lo que no se desagrega por grupo (se marca con guion). La clasificación es por exposición fiscal neta al precio del petróleo, no por producción: en los exportadores netos el alza del Brent infla la renta petrolera que financia el subsidio, mientras que en los importadores netos encarece el costo de suministro y agrava el gasto. Fuente: IMF Fossil Fuel Subsidies Database; precio Brent: EIA.</t>
+    <t xml:space="preserve">Notas. Estadística descriptiva de las variables del análisis para el panel de 34 países de América Latina y el Caribe, 2015-2023. Cada celda reporta la media y, entre paréntesis, la desviación estándar de las observaciones país-año del grupo. El subsidio explícito es la brecha entre el precio al consumidor y el costo de suministro; el implícito añade las externalidades no internalizadas y el IVA no aplicado; el total es la suma de ambos. El subsidio implícito y el total tienen menor cobertura (no estimados para todos los país-año). El análisis del choque (Figuras 1 y 2) se concentra en el componente explícito por ser el más sensible al precio internacional en el corto plazo: reacciona de forma directa cuando el alza del costo de suministro no se traslada al precio al consumidor. El implícito depende del volumen consumido y de parámetros de daño ambiental, no del precio del petróleo, por lo que apenas responde al choque en el corto plazo. El precio del Brent (Panel B) es la serie internacional, común a todos los países cada año, por lo que no se desagrega por grupo (se marca con guion). La clasificación es por exposición fiscal neta al precio del petróleo, no por producción: en los exportadores netos el alza del Brent infla la renta petrolera que financia el subsidio, mientras que en los importadores netos encarece el costo de suministro y agrava el gasto. Fuente: IMF Fossil Fuel Subsidies Database; precio Brent: EIA.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="166" formatCode="@"/>
     <numFmt numFmtId="167" formatCode="@"/>
     <numFmt numFmtId="168" formatCode="0"/>
-    <numFmt numFmtId="169" formatCode="0"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -254,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -282,9 +218,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -691,125 +624,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" ht="326" customHeight="1">
+      <c r="B10" s="11" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>34</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" ht="368" customHeight="1">
-      <c r="B17" s="12" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B10:E10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>